<commit_message>
removed unessesary resturants. added 73. removed "view ad prices" button.
</commit_message>
<xml_diff>
--- a/restaurant_data.xlsx
+++ b/restaurant_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maail_02624\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dhiraagu-my.sharepoint.com/personal/maail_02624_dhiraagu_com_mv/Documents/personal/websites/roadhaonline/ramadan_menu/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72363FA6-3B68-497B-9D03-D2EA87BA25B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{72363FA6-3B68-497B-9D03-D2EA87BA25B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D933DD18-B49B-4E81-BF42-7B58EE1834C4}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="759" xr2:uid="{D14014FB-EFB2-4719-9A66-74152C34B487}"/>
+    <workbookView xWindow="-19310" yWindow="3730" windowWidth="19420" windowHeight="11500" tabRatio="759" xr2:uid="{D14014FB-EFB2-4719-9A66-74152C34B487}"/>
   </bookViews>
   <sheets>
     <sheet name="restaurant_list" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1977" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1962" uniqueCount="249">
   <si>
     <t>Nuts / Water</t>
   </si>
@@ -743,42 +743,6 @@
     <t>sheet_name</t>
   </si>
   <si>
-    <t>mamak</t>
-  </si>
-  <si>
-    <t>images/mamak/mamak_logo.png</t>
-  </si>
-  <si>
-    <t>images/mamak/mamak_banner.png</t>
-  </si>
-  <si>
-    <t>citron</t>
-  </si>
-  <si>
-    <t>images/citron/citron_logo.png</t>
-  </si>
-  <si>
-    <t>images/citron/citron_banner.png</t>
-  </si>
-  <si>
-    <t>house of flavors</t>
-  </si>
-  <si>
-    <t>Acha's Poppadums</t>
-  </si>
-  <si>
-    <t>images/house_of_flavors/house_of_flavors_logo.png</t>
-  </si>
-  <si>
-    <t>images/house_of_flavors/house_of_flavors_banner.png</t>
-  </si>
-  <si>
-    <t>images/acha's_poppodums/acha's_poppodums_logo.png</t>
-  </si>
-  <si>
-    <t>images/acha's_poppodums/acha's_poppodums_banner.png</t>
-  </si>
-  <si>
     <t>restaurant_name</t>
   </si>
   <si>
@@ -822,6 +786,9 @@
   </si>
   <si>
     <t>DATES</t>
+  </si>
+  <si>
+    <t>images/73/73_logo.png</t>
   </si>
 </sst>
 </file>
@@ -863,11 +830,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1202,7 +1170,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CA06C4E-D4C8-4C24-9F63-95F191572C1F}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.81640625" customWidth="1"/>
@@ -1211,88 +1179,43 @@
     <col min="4" max="4" width="18.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>245</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>246</v>
-      </c>
-      <c r="B2" t="s">
-        <v>247</v>
-      </c>
-      <c r="C2" t="s">
+    <row r="2" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>73</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="D2" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>233</v>
-      </c>
-      <c r="B3" t="s">
-        <v>234</v>
-      </c>
-      <c r="C3" t="s">
-        <v>235</v>
-      </c>
-      <c r="D3" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>236</v>
-      </c>
-      <c r="B4" t="s">
-        <v>237</v>
-      </c>
-      <c r="C4" t="s">
-        <v>238</v>
-      </c>
-      <c r="D4" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>239</v>
-      </c>
-      <c r="B5" t="s">
-        <v>241</v>
-      </c>
-      <c r="C5" t="s">
-        <v>242</v>
-      </c>
-      <c r="D5" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>240</v>
-      </c>
-      <c r="B6" t="s">
-        <v>243</v>
-      </c>
-      <c r="C6" t="s">
-        <v>244</v>
-      </c>
-      <c r="D6" t="s">
-        <v>240</v>
+      <c r="D3" s="2">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1334,7 +1257,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="D2">
         <v>200</v>
@@ -1359,7 +1282,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -1370,7 +1293,7 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -1381,7 +1304,7 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -1392,7 +1315,7 @@
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -1403,7 +1326,7 @@
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -1414,7 +1337,7 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -1425,7 +1348,7 @@
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -1436,7 +1359,7 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -1447,7 +1370,7 @@
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
@@ -1458,7 +1381,7 @@
         <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="D14">
         <v>200</v>
@@ -1483,7 +1406,7 @@
         <v>6</v>
       </c>
       <c r="C16" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
@@ -1494,7 +1417,7 @@
         <v>8</v>
       </c>
       <c r="C17" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
@@ -1505,7 +1428,7 @@
         <v>8</v>
       </c>
       <c r="C18" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
@@ -1516,7 +1439,7 @@
         <v>8</v>
       </c>
       <c r="C19" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
@@ -1527,7 +1450,7 @@
         <v>8</v>
       </c>
       <c r="C20" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
@@ -1538,7 +1461,7 @@
         <v>8</v>
       </c>
       <c r="C21" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
@@ -1549,7 +1472,7 @@
         <v>8</v>
       </c>
       <c r="C22" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
@@ -1560,7 +1483,7 @@
         <v>8</v>
       </c>
       <c r="C23" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
@@ -1571,7 +1494,7 @@
         <v>8</v>
       </c>
       <c r="C24" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
@@ -1582,7 +1505,7 @@
         <v>4</v>
       </c>
       <c r="C26" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="D26">
         <v>200</v>
@@ -1607,7 +1530,7 @@
         <v>6</v>
       </c>
       <c r="C28" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
@@ -1618,7 +1541,7 @@
         <v>8</v>
       </c>
       <c r="C29" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
@@ -1629,7 +1552,7 @@
         <v>8</v>
       </c>
       <c r="C30" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
@@ -1640,7 +1563,7 @@
         <v>8</v>
       </c>
       <c r="C31" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
@@ -1651,7 +1574,7 @@
         <v>8</v>
       </c>
       <c r="C32" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
@@ -1662,7 +1585,7 @@
         <v>8</v>
       </c>
       <c r="C33" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
@@ -1673,7 +1596,7 @@
         <v>8</v>
       </c>
       <c r="C34" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
@@ -1684,7 +1607,7 @@
         <v>8</v>
       </c>
       <c r="C35" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
@@ -1695,7 +1618,7 @@
         <v>8</v>
       </c>
       <c r="C36" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
@@ -1706,7 +1629,7 @@
         <v>4</v>
       </c>
       <c r="C38" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="D38">
         <v>200</v>
@@ -1731,7 +1654,7 @@
         <v>6</v>
       </c>
       <c r="C40" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
@@ -1742,7 +1665,7 @@
         <v>8</v>
       </c>
       <c r="C41" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
@@ -1753,7 +1676,7 @@
         <v>8</v>
       </c>
       <c r="C42" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
@@ -1764,7 +1687,7 @@
         <v>8</v>
       </c>
       <c r="C43" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
@@ -1775,7 +1698,7 @@
         <v>8</v>
       </c>
       <c r="C44" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
@@ -1786,7 +1709,7 @@
         <v>8</v>
       </c>
       <c r="C45" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
@@ -1797,7 +1720,7 @@
         <v>8</v>
       </c>
       <c r="C46" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
@@ -1808,7 +1731,7 @@
         <v>8</v>
       </c>
       <c r="C47" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
@@ -1819,7 +1742,7 @@
         <v>8</v>
       </c>
       <c r="C48" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
@@ -1830,7 +1753,7 @@
         <v>4</v>
       </c>
       <c r="C56" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="D56">
         <v>200</v>
@@ -1855,7 +1778,7 @@
         <v>6</v>
       </c>
       <c r="C58" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
@@ -1866,7 +1789,7 @@
         <v>8</v>
       </c>
       <c r="C59" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
@@ -1877,7 +1800,7 @@
         <v>8</v>
       </c>
       <c r="C60" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
@@ -1888,7 +1811,7 @@
         <v>8</v>
       </c>
       <c r="C61" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
@@ -1899,7 +1822,7 @@
         <v>8</v>
       </c>
       <c r="C62" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
@@ -1910,7 +1833,7 @@
         <v>8</v>
       </c>
       <c r="C63" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
@@ -1921,7 +1844,7 @@
         <v>8</v>
       </c>
       <c r="C64" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
@@ -1932,7 +1855,7 @@
         <v>8</v>
       </c>
       <c r="C65" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
@@ -1943,7 +1866,7 @@
         <v>8</v>
       </c>
       <c r="C66" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
@@ -1954,7 +1877,7 @@
         <v>4</v>
       </c>
       <c r="C68" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="D68">
         <v>200</v>
@@ -1979,7 +1902,7 @@
         <v>6</v>
       </c>
       <c r="C70" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
@@ -1990,7 +1913,7 @@
         <v>8</v>
       </c>
       <c r="C71" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
@@ -2001,7 +1924,7 @@
         <v>8</v>
       </c>
       <c r="C72" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
@@ -2012,7 +1935,7 @@
         <v>8</v>
       </c>
       <c r="C73" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
@@ -2023,7 +1946,7 @@
         <v>8</v>
       </c>
       <c r="C74" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
@@ -2034,7 +1957,7 @@
         <v>8</v>
       </c>
       <c r="C75" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
@@ -2045,7 +1968,7 @@
         <v>8</v>
       </c>
       <c r="C76" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
@@ -2056,7 +1979,7 @@
         <v>8</v>
       </c>
       <c r="C77" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
@@ -2067,7 +1990,7 @@
         <v>8</v>
       </c>
       <c r="C78" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
@@ -2078,7 +2001,7 @@
         <v>4</v>
       </c>
       <c r="C80" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="D80">
         <v>200</v>
@@ -2103,7 +2026,7 @@
         <v>6</v>
       </c>
       <c r="C82" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.35">
@@ -2114,7 +2037,7 @@
         <v>8</v>
       </c>
       <c r="C83" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.35">
@@ -2125,7 +2048,7 @@
         <v>8</v>
       </c>
       <c r="C84" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.35">
@@ -2136,7 +2059,7 @@
         <v>8</v>
       </c>
       <c r="C85" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.35">
@@ -2147,7 +2070,7 @@
         <v>8</v>
       </c>
       <c r="C86" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.35">
@@ -2158,7 +2081,7 @@
         <v>8</v>
       </c>
       <c r="C87" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.35">
@@ -2169,7 +2092,7 @@
         <v>8</v>
       </c>
       <c r="C88" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.35">
@@ -2180,7 +2103,7 @@
         <v>8</v>
       </c>
       <c r="C89" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.35">
@@ -2191,7 +2114,7 @@
         <v>8</v>
       </c>
       <c r="C90" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated 73 logo to latest and menu to "under consturction"
</commit_message>
<xml_diff>
--- a/restaurant_data.xlsx
+++ b/restaurant_data.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dhiraagu-my.sharepoint.com/personal/maail_02624_dhiraagu_com_mv/Documents/personal/websites/roadhaonline/ramadan_menu/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{72363FA6-3B68-497B-9D03-D2EA87BA25B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D933DD18-B49B-4E81-BF42-7B58EE1834C4}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{72363FA6-3B68-497B-9D03-D2EA87BA25B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD52EB1A-FA80-4316-A3DB-9FFE470BC589}"/>
   <bookViews>
     <workbookView xWindow="-19310" yWindow="3730" windowWidth="19420" windowHeight="11500" tabRatio="759" xr2:uid="{D14014FB-EFB2-4719-9A66-74152C34B487}"/>
   </bookViews>
   <sheets>
     <sheet name="restaurant_list" sheetId="1" r:id="rId1"/>
-    <sheet name="koththu hut" sheetId="9" r:id="rId2"/>
-    <sheet name="mamak" sheetId="2" r:id="rId3"/>
-    <sheet name="citron" sheetId="3" r:id="rId4"/>
-    <sheet name="house of flavors" sheetId="6" r:id="rId5"/>
-    <sheet name="Acha's Poppadums" sheetId="7" r:id="rId6"/>
-    <sheet name="ny steak shack" sheetId="8" r:id="rId7"/>
+    <sheet name="73" sheetId="10" r:id="rId2"/>
+    <sheet name="koththu hut" sheetId="9" r:id="rId3"/>
+    <sheet name="mamak" sheetId="2" r:id="rId4"/>
+    <sheet name="citron" sheetId="3" r:id="rId5"/>
+    <sheet name="house of flavors" sheetId="6" r:id="rId6"/>
+    <sheet name="Acha's Poppadums" sheetId="7" r:id="rId7"/>
+    <sheet name="ny steak shack" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1962" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1975" uniqueCount="252">
   <si>
     <t>Nuts / Water</t>
   </si>
@@ -788,14 +789,23 @@
     <t>DATES</t>
   </si>
   <si>
-    <t>images/73/73_logo.png</t>
+    <t>images/73/73_logo.jpeg</t>
+  </si>
+  <si>
+    <t>UNDER CONSTRUCTION</t>
+  </si>
+  <si>
+    <t>we will be uploading the true menu soon</t>
+  </si>
+  <si>
+    <t>images/under_construction.png</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -808,6 +818,12 @@
       <color theme="1"/>
       <name val="Helvetica"/>
       <family val="18"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -830,12 +846,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -851,6 +866,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1179,42 +1198,45 @@
     <col min="4" max="4" width="18.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>233</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>230</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>231</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>234</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>235</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" t="s">
         <v>236</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
         <v>73</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>248</v>
       </c>
-      <c r="D3" s="2">
+      <c r="C3" t="s">
+        <v>251</v>
+      </c>
+      <c r="D3">
         <v>73</v>
       </c>
     </row>
@@ -1225,6 +1247,72 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B203C57B-5E1D-4952-8C96-E88B3FA9DAD6}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="20.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{914D9201-C41D-4512-A19F-3E2E6A2C8E63}">
   <dimension ref="A1:D90"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2122,7 +2210,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74F297DF-EE82-4C46-A8A1-7FFBDBE8DB35}">
   <dimension ref="A1:D131"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3535,7 +3623,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72118D6-E8F8-4575-9467-81BC74209E5B}">
   <dimension ref="A1:D220"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -5917,7 +6005,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9ACDF15-8D27-4E0A-A148-197DCB9A4BBC}">
   <dimension ref="A1:D92"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -6969,7 +7057,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A907F4E-741D-4896-A5D4-50E4A970A72D}">
   <dimension ref="A1:D134"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -8486,7 +8574,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15FD1D32-DA8B-4619-A76E-9545BAC189FD}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>